<commit_message>
Added visuals to food effects, implementation and bug fixing
</commit_message>
<xml_diff>
--- a/Food Progression.xlsx
+++ b/Food Progression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Nutri Mayhem\NutriCrush-Unity-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87CE47D8-427D-42E4-B3FE-DDA6CF07E71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA98762-EE3C-498C-9527-17FE9498C110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8110" yWindow="3210" windowWidth="21600" windowHeight="14680" activeTab="1" xr2:uid="{3A71858E-782A-488A-BF56-898FF2A6D53B}"/>
   </bookViews>
@@ -435,9 +435,6 @@
     <t>Random Effects</t>
   </si>
   <si>
-    <t>Shared Health</t>
-  </si>
-  <si>
     <t>Cherries</t>
   </si>
   <si>
@@ -505,6 +502,9 @@
   </si>
   <si>
     <t>Slow Release</t>
+  </si>
+  <si>
+    <t>Max Cards</t>
   </si>
 </sst>
 </file>
@@ -994,26 +994,25 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1435,2512 +1434,2512 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2">
         <v>30</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2">
         <v>0.2</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2">
         <v>0.05</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2">
         <v>3.4</v>
       </c>
-      <c r="H2" s="8">
+      <c r="H2">
         <v>0</v>
       </c>
-      <c r="I2" s="8">
-        <v>3</v>
-      </c>
-      <c r="J2" s="8">
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
         <v>10</v>
       </c>
-      <c r="K2" s="8">
+      <c r="K2">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3">
         <v>78</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3">
         <v>3.4</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3">
         <v>6.2E-2</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3">
         <v>0.6</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3">
         <v>1.6</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3">
         <v>4</v>
       </c>
-      <c r="J3" s="8">
+      <c r="J3">
         <v>8</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="8">
-        <v>3</v>
-      </c>
-      <c r="B4" s="8" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4">
         <v>42</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="8">
-        <v>3</v>
-      </c>
-      <c r="F4" s="8">
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4">
         <v>5</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4">
         <v>0.6</v>
       </c>
-      <c r="I4" s="8">
-        <v>3</v>
-      </c>
-      <c r="J4" s="8">
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4">
         <v>11</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5">
         <v>165</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5">
         <v>3.6</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5">
         <v>0.08</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5">
         <v>1</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5">
         <v>2</v>
       </c>
-      <c r="J5" s="8">
+      <c r="J5">
         <v>8</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="8">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6">
         <v>75</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6">
         <v>0.8</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6">
         <v>0.14000000000000001</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6">
         <v>1.5</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6">
         <v>0.2</v>
       </c>
-      <c r="I6" s="8">
-        <v>3</v>
-      </c>
-      <c r="J6" s="8">
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
         <v>2</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7">
         <v>158</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7">
         <v>0.5</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7">
         <v>3.4000000000000002E-2</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7">
         <v>0.8</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7">
         <v>0.1</v>
       </c>
-      <c r="I7" s="8">
+      <c r="I7">
         <v>2</v>
       </c>
-      <c r="J7" s="8">
-        <v>3</v>
-      </c>
-      <c r="K7" s="8">
+      <c r="J7">
+        <v>3</v>
+      </c>
+      <c r="K7">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="8">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8">
         <v>206</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8">
         <v>9.6</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8">
         <v>0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8">
         <v>2.4</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8">
         <v>2</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8">
         <v>10</v>
       </c>
-      <c r="K8" s="8">
+      <c r="K8">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9">
         <v>112</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9">
         <v>3.37</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9">
         <v>0.17</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9">
         <v>0.15</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9">
         <v>4</v>
       </c>
-      <c r="I9" s="8">
-        <v>3</v>
-      </c>
-      <c r="J9" s="8">
+      <c r="I9">
+        <v>3</v>
+      </c>
+      <c r="J9">
         <v>10</v>
       </c>
-      <c r="K9" s="8">
+      <c r="K9">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10">
         <v>45</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10">
         <v>2</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10">
         <v>0.32</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10">
         <v>0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10">
         <v>1</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10">
         <v>2</v>
       </c>
-      <c r="J10" s="8">
-        <v>3</v>
-      </c>
-      <c r="K10" s="8">
+      <c r="J10">
+        <v>3</v>
+      </c>
+      <c r="K10">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="8">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11">
         <v>130</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11">
         <v>0.3</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11">
         <v>1E-3</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11">
         <v>0.1</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11">
         <v>0.1</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11">
         <v>5</v>
       </c>
-      <c r="J11" s="8">
+      <c r="J11">
         <v>2</v>
       </c>
-      <c r="K11" s="8">
+      <c r="K11">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="8">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12">
         <v>100</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12">
         <v>2</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12">
         <v>0</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12">
         <v>1</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12">
         <v>0.2</v>
       </c>
-      <c r="I12" s="8">
-        <v>3</v>
-      </c>
-      <c r="J12" s="8">
-        <v>3</v>
-      </c>
-      <c r="K12" s="8">
+      <c r="I12">
+        <v>3</v>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+      <c r="K12">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="8">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13">
         <v>160</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13">
         <v>0.2</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13">
         <v>2.4E-2</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13">
         <v>1.2</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13">
         <v>0.1</v>
       </c>
-      <c r="I13" s="8">
-        <v>3</v>
-      </c>
-      <c r="J13" s="8">
+      <c r="I13">
+        <v>3</v>
+      </c>
+      <c r="J13">
         <v>2</v>
       </c>
-      <c r="K13" s="8">
+      <c r="K13">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="8">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14">
         <v>116</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14">
         <v>0.4</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14">
         <v>2E-3</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14">
         <v>1.8</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14">
         <v>0.1</v>
       </c>
-      <c r="I14" s="8">
+      <c r="I14">
         <v>5</v>
       </c>
-      <c r="J14" s="8">
+      <c r="J14">
         <v>16</v>
       </c>
-      <c r="K14" s="8">
+      <c r="K14">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="8">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15">
         <v>84</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15">
         <v>0.8</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15">
         <v>0.1</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15">
         <v>5</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15">
         <v>0.1</v>
       </c>
-      <c r="I15" s="8">
-        <v>3</v>
-      </c>
-      <c r="J15" s="8">
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
         <v>9</v>
       </c>
-      <c r="K15" s="8">
+      <c r="K15">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="8">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16">
         <v>250</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16">
         <v>15</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16">
         <v>0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16">
         <v>6.8</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16">
         <v>2</v>
       </c>
-      <c r="J16" s="8">
-        <v>3</v>
-      </c>
-      <c r="K16" s="8">
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="8">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17">
         <v>242</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17">
         <v>14</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17">
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17">
         <v>0</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17">
         <v>7.7</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17">
         <v>2</v>
       </c>
-      <c r="J17" s="8">
-        <v>3</v>
-      </c>
-      <c r="K17" s="8">
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="8">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18">
         <v>34</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18">
         <v>0.4</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18">
         <v>1.7</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18">
         <v>0.1</v>
       </c>
-      <c r="I18" s="8">
-        <v>3</v>
-      </c>
-      <c r="J18" s="8">
+      <c r="I18">
+        <v>3</v>
+      </c>
+      <c r="J18">
         <v>16</v>
       </c>
-      <c r="K18" s="8">
+      <c r="K18">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="8">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19">
         <v>23</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" t="s">
         <v>30</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E19">
         <v>0.4</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19">
         <v>9.7000000000000003E-2</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19">
         <v>0.4</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19">
         <v>0.1</v>
       </c>
-      <c r="I19" s="8">
+      <c r="I19">
         <v>2</v>
       </c>
-      <c r="J19" s="8">
+      <c r="J19">
         <v>16</v>
       </c>
-      <c r="K19" s="8">
+      <c r="K19">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="8">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20">
         <v>18</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" t="s">
         <v>31</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20">
         <v>0.2</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F20">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20">
         <v>2.6</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20">
         <v>0</v>
       </c>
-      <c r="I20" s="8">
-        <v>3</v>
-      </c>
-      <c r="J20" s="8">
+      <c r="I20">
+        <v>3</v>
+      </c>
+      <c r="J20">
         <v>11</v>
       </c>
-      <c r="K20" s="8">
+      <c r="K20">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="8">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21">
         <v>164</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21">
         <v>2.4</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F21">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21">
         <v>4.8</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21">
         <v>0.4</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21">
         <v>5</v>
       </c>
-      <c r="J21" s="8">
+      <c r="J21">
         <v>10</v>
       </c>
-      <c r="K21" s="8">
+      <c r="K21">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="8">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22">
         <v>89</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E22">
         <v>0.3</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F22">
         <v>1E-3</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22">
         <v>12</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22">
         <v>0.1</v>
       </c>
-      <c r="I22" s="8">
-        <v>3</v>
-      </c>
-      <c r="J22" s="8">
+      <c r="I22">
+        <v>3</v>
+      </c>
+      <c r="J22">
         <v>2</v>
       </c>
-      <c r="K22" s="8">
+      <c r="K22">
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="8">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23">
         <v>160</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23">
         <v>12</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23">
         <v>0.7</v>
       </c>
-      <c r="H23" s="8">
+      <c r="H23">
         <v>2</v>
       </c>
-      <c r="I23" s="8">
+      <c r="I23">
         <v>2</v>
       </c>
-      <c r="J23" s="8">
+      <c r="J23">
         <v>16</v>
       </c>
-      <c r="K23" s="8">
+      <c r="K23">
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="8">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24">
         <v>30</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24">
         <v>0.4</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24">
         <v>0.01</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24">
         <v>0</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24">
         <v>0</v>
       </c>
-      <c r="I24" s="8">
-        <v>3</v>
-      </c>
-      <c r="J24" s="8">
+      <c r="I24">
+        <v>3</v>
+      </c>
+      <c r="J24">
         <v>8</v>
       </c>
-      <c r="K24" s="8">
+      <c r="K24">
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="8">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" t="s">
         <v>36</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25">
         <v>17</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25">
         <v>0.2</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25">
         <v>1E-3</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25">
         <v>2.5</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25">
         <v>0.1</v>
       </c>
-      <c r="I25" s="8">
+      <c r="I25">
         <v>4</v>
       </c>
-      <c r="J25" s="8">
+      <c r="J25">
         <v>11</v>
       </c>
-      <c r="K25" s="8">
+      <c r="K25">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="8">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26">
         <v>127</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26">
         <v>0.4</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26">
         <v>2E-3</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26">
         <v>0.3</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26">
         <v>0.1</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26">
         <v>5</v>
       </c>
-      <c r="J26" s="8">
+      <c r="J26">
         <v>9</v>
       </c>
-      <c r="K26" s="8">
+      <c r="K26">
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="8">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27">
         <v>52</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" t="s">
         <v>39</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27">
         <v>0.2</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27">
         <v>1E-3</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27">
         <v>10</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27">
         <v>0</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27">
         <v>4</v>
       </c>
-      <c r="J27" s="8">
-        <v>3</v>
-      </c>
-      <c r="K27" s="8">
+      <c r="J27">
+        <v>3</v>
+      </c>
+      <c r="K27">
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="8">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28">
         <v>39</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" t="s">
         <v>40</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28">
         <v>0.25</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28">
         <v>6.6</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28">
         <v>0.02</v>
       </c>
-      <c r="I28" s="8">
-        <v>3</v>
-      </c>
-      <c r="J28" s="8">
+      <c r="I28">
+        <v>3</v>
+      </c>
+      <c r="J28">
         <v>11</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28">
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="8">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" t="s">
         <v>41</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29">
         <v>25</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" t="s">
         <v>41</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29">
         <v>0.3</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29">
         <v>0.03</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29">
         <v>1.9</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29">
         <v>0</v>
       </c>
-      <c r="I29" s="8">
-        <v>3</v>
-      </c>
-      <c r="J29" s="8">
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
         <v>16</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29">
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="8">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30">
         <v>30</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" t="s">
         <v>42</v>
       </c>
-      <c r="E30" s="8">
+      <c r="E30">
         <v>0.3</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F30">
         <v>0.04</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30">
         <v>4.4000000000000004</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30">
         <v>0</v>
       </c>
-      <c r="I30" s="8">
-        <v>3</v>
-      </c>
-      <c r="J30" s="8">
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
         <v>8</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30">
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="8">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C31">
         <v>208</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" t="s">
         <v>43</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31">
         <v>9</v>
       </c>
-      <c r="F31" s="8">
+      <c r="F31">
         <v>0.3</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31">
         <v>0</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31">
         <v>1.5</v>
       </c>
-      <c r="I31" s="8">
+      <c r="I31">
         <v>2</v>
       </c>
-      <c r="J31" s="8">
+      <c r="J31">
         <v>9</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="8">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" t="s">
         <v>44</v>
       </c>
-      <c r="C32" s="8">
+      <c r="C32">
         <v>115</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E32">
         <v>2</v>
       </c>
-      <c r="F32" s="8">
+      <c r="F32">
         <v>0.5</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32">
         <v>0</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32">
         <v>1</v>
       </c>
-      <c r="I32" s="8">
+      <c r="I32">
         <v>2</v>
       </c>
-      <c r="J32" s="8">
+      <c r="J32">
         <v>10</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="8">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" t="s">
         <v>45</v>
       </c>
-      <c r="C33" s="8">
+      <c r="C33">
         <v>17</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" t="s">
         <v>45</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E33">
         <v>0.3</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33">
         <v>1.2E-2</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33">
         <v>2</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33">
         <v>0</v>
       </c>
-      <c r="I33" s="8">
-        <v>3</v>
-      </c>
-      <c r="J33" s="8">
+      <c r="I33">
+        <v>3</v>
+      </c>
+      <c r="J33">
         <v>11</v>
       </c>
-      <c r="K33" s="8">
+      <c r="K33">
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="8">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" t="s">
         <v>46</v>
       </c>
-      <c r="C34" s="8">
+      <c r="C34">
         <v>40</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D34" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="8">
+      <c r="E34">
         <v>0.2</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F34">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34">
         <v>4.2</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34">
         <v>0</v>
       </c>
-      <c r="I34" s="8">
+      <c r="I34">
         <v>4</v>
       </c>
-      <c r="J34" s="8">
+      <c r="J34">
         <v>8</v>
       </c>
-      <c r="K34" s="8">
+      <c r="K34">
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="8">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35">
         <v>60</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="D35" t="s">
         <v>47</v>
       </c>
-      <c r="E35" s="8">
+      <c r="E35">
         <v>1.5</v>
       </c>
-      <c r="F35" s="8">
+      <c r="F35">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="G35" s="8">
+      <c r="G35">
         <v>6</v>
       </c>
-      <c r="H35" s="8">
+      <c r="H35">
         <v>2</v>
       </c>
-      <c r="I35" s="8">
+      <c r="I35">
         <v>4</v>
       </c>
-      <c r="J35" s="8">
+      <c r="J35">
         <v>11</v>
       </c>
-      <c r="K35" s="8">
+      <c r="K35">
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="8">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="8">
+      <c r="C36">
         <v>180</v>
       </c>
-      <c r="D36" s="8" t="s">
+      <c r="D36" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="8">
+      <c r="E36">
         <v>13</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F36">
         <v>0.2</v>
       </c>
-      <c r="G36" s="8">
+      <c r="G36">
         <v>2</v>
       </c>
-      <c r="H36" s="8">
+      <c r="H36">
         <v>2</v>
       </c>
-      <c r="I36" s="8">
+      <c r="I36">
         <v>5</v>
       </c>
-      <c r="J36" s="8">
+      <c r="J36">
         <v>2</v>
       </c>
-      <c r="K36" s="8">
+      <c r="K36">
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="8">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A37">
         <v>37</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" t="s">
         <v>49</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37">
         <v>200</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" t="s">
         <v>49</v>
       </c>
-      <c r="E37" s="8">
+      <c r="E37">
         <v>5</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37">
         <v>0.03</v>
       </c>
-      <c r="G37" s="8">
+      <c r="G37">
         <v>15</v>
       </c>
-      <c r="H37" s="8">
+      <c r="H37">
         <v>11</v>
       </c>
-      <c r="I37" s="8">
+      <c r="I37">
         <v>4</v>
       </c>
-      <c r="J37" s="8">
+      <c r="J37">
         <v>2</v>
       </c>
-      <c r="K37" s="8">
+      <c r="K37">
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="8">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A38">
         <v>39</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" t="s">
         <v>50</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38">
         <v>73</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" t="s">
         <v>50</v>
       </c>
-      <c r="E38" s="8">
+      <c r="E38">
         <v>0.2</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="G38" s="8">
+      <c r="G38">
         <v>9</v>
       </c>
-      <c r="H38" s="8">
+      <c r="H38">
         <v>0</v>
       </c>
-      <c r="I38" s="8">
-        <v>3</v>
-      </c>
-      <c r="J38" s="8">
-        <v>3</v>
-      </c>
-      <c r="K38" s="8">
+      <c r="I38">
+        <v>3</v>
+      </c>
+      <c r="J38">
+        <v>3</v>
+      </c>
+      <c r="K38">
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="8">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39">
         <v>40</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" t="s">
         <v>51</v>
       </c>
-      <c r="C39" s="8">
+      <c r="C39">
         <v>119</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="D39" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="8">
+      <c r="E39">
         <v>1.5</v>
       </c>
-      <c r="F39" s="8">
+      <c r="F39">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="G39" s="8">
+      <c r="G39">
         <v>0</v>
       </c>
-      <c r="H39" s="8">
+      <c r="H39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="I39" s="8">
+      <c r="I39">
         <v>2</v>
       </c>
-      <c r="J39" s="8">
-        <v>3</v>
-      </c>
-      <c r="K39" s="8">
+      <c r="J39">
+        <v>3</v>
+      </c>
+      <c r="K39">
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="8">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A40">
         <v>41</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="8">
+      <c r="C40">
         <v>120</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="D40" t="s">
         <v>52</v>
       </c>
-      <c r="E40" s="8">
+      <c r="E40">
         <v>0.5</v>
       </c>
-      <c r="F40" s="8">
+      <c r="F40">
         <v>0.14000000000000001</v>
       </c>
-      <c r="G40" s="8">
+      <c r="G40">
         <v>0</v>
       </c>
-      <c r="H40" s="8">
+      <c r="H40">
         <v>0.8</v>
       </c>
-      <c r="I40" s="8">
-        <v>3</v>
-      </c>
-      <c r="J40" s="8">
+      <c r="I40">
+        <v>3</v>
+      </c>
+      <c r="J40">
         <v>10</v>
       </c>
-      <c r="K40" s="8">
+      <c r="K40">
         <v>30</v>
       </c>
     </row>
-    <row r="41" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="8">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41">
         <v>42</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" t="s">
         <v>53</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41">
         <v>75</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="D41" t="s">
         <v>53</v>
       </c>
-      <c r="E41" s="8">
+      <c r="E41">
         <v>1.8</v>
       </c>
-      <c r="F41" s="8">
+      <c r="F41">
         <v>0.26</v>
       </c>
-      <c r="G41" s="8">
+      <c r="G41">
         <v>0.5</v>
       </c>
-      <c r="H41" s="8">
+      <c r="H41">
         <v>0</v>
       </c>
-      <c r="I41" s="8">
+      <c r="I41">
         <v>2</v>
       </c>
-      <c r="J41" s="8">
+      <c r="J41">
         <v>9</v>
       </c>
-      <c r="K41" s="8">
+      <c r="K41">
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="8">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A42">
         <v>43</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" t="s">
         <v>54</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C42">
         <v>68</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="D42" t="s">
         <v>54</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E42">
         <v>0.2</v>
       </c>
-      <c r="F42" s="8">
+      <c r="F42">
         <v>2E-3</v>
       </c>
-      <c r="G42" s="8">
+      <c r="G42">
         <v>15</v>
       </c>
-      <c r="H42" s="8">
+      <c r="H42">
         <v>0.1</v>
       </c>
-      <c r="I42" s="8">
+      <c r="I42">
         <v>4</v>
       </c>
-      <c r="J42" s="8">
+      <c r="J42">
         <v>11</v>
       </c>
-      <c r="K42" s="8">
+      <c r="K42">
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="8">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A43">
         <v>45</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43">
         <v>32</v>
       </c>
-      <c r="D43" s="8" t="s">
+      <c r="D43" t="s">
         <v>55</v>
       </c>
-      <c r="E43" s="8">
+      <c r="E43">
         <v>0.3</v>
       </c>
-      <c r="F43" s="8">
+      <c r="F43">
         <v>1E-3</v>
       </c>
-      <c r="G43" s="8">
+      <c r="G43">
         <v>4.9000000000000004</v>
       </c>
-      <c r="H43" s="8">
+      <c r="H43">
         <v>0</v>
       </c>
-      <c r="I43" s="8">
+      <c r="I43">
         <v>2</v>
       </c>
-      <c r="J43" s="8">
+      <c r="J43">
         <v>11</v>
       </c>
-      <c r="K43" s="8">
+      <c r="K43">
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="8">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A44">
         <v>46</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" t="s">
         <v>56</v>
       </c>
-      <c r="C44" s="8">
+      <c r="C44">
         <v>250</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" t="s">
         <v>56</v>
       </c>
-      <c r="E44" s="8">
+      <c r="E44">
         <v>12</v>
       </c>
-      <c r="F44" s="8">
+      <c r="F44">
         <v>0.2</v>
       </c>
-      <c r="G44" s="8">
+      <c r="G44">
         <v>25</v>
       </c>
-      <c r="H44" s="8">
+      <c r="H44">
         <v>5</v>
       </c>
-      <c r="I44" s="8">
-        <v>3</v>
-      </c>
-      <c r="J44" s="8">
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
         <v>2</v>
       </c>
-      <c r="K44" s="8">
+      <c r="K44">
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="8">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A45">
         <v>49</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" t="s">
         <v>57</v>
       </c>
-      <c r="C45" s="8">
+      <c r="C45">
         <v>56</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D45" t="s">
         <v>57</v>
       </c>
-      <c r="E45" s="8">
+      <c r="E45">
         <v>0</v>
       </c>
-      <c r="F45" s="8">
+      <c r="F45">
         <v>0.08</v>
       </c>
-      <c r="G45" s="8">
+      <c r="G45">
         <v>10</v>
       </c>
-      <c r="H45" s="8">
+      <c r="H45">
         <v>0</v>
       </c>
-      <c r="I45" s="8">
+      <c r="I45">
         <v>5</v>
       </c>
-      <c r="J45" s="8">
+      <c r="J45">
         <v>2</v>
       </c>
-      <c r="K45" s="8">
+      <c r="K45">
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="8">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A46">
         <v>50</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="B46" t="s">
         <v>58</v>
       </c>
-      <c r="C46" s="8">
+      <c r="C46">
         <v>80</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="D46" t="s">
         <v>58</v>
       </c>
-      <c r="E46" s="8">
+      <c r="E46">
         <v>4</v>
       </c>
-      <c r="F46" s="8">
+      <c r="F46">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="G46" s="8">
+      <c r="G46">
         <v>1.5</v>
       </c>
-      <c r="H46" s="8">
+      <c r="H46">
         <v>0</v>
       </c>
-      <c r="I46" s="8">
-        <v>3</v>
-      </c>
-      <c r="J46" s="8">
+      <c r="I46">
+        <v>3</v>
+      </c>
+      <c r="J46">
         <v>8</v>
       </c>
-      <c r="K46" s="8">
+      <c r="K46">
         <v>30</v>
       </c>
     </row>
-    <row r="47" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="8">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A47">
         <v>51</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B47" t="s">
         <v>109</v>
       </c>
-      <c r="C47" s="8">
+      <c r="C47">
         <v>90</v>
       </c>
-      <c r="D47" s="8" t="s">
+      <c r="D47" t="s">
         <v>109</v>
       </c>
-      <c r="E47" s="8">
+      <c r="E47">
         <v>13</v>
       </c>
-      <c r="F47" s="8">
+      <c r="F47">
         <v>0</v>
       </c>
-      <c r="G47" s="8">
+      <c r="G47">
         <v>1.2</v>
       </c>
-      <c r="H47" s="8">
+      <c r="H47">
         <v>1</v>
       </c>
-      <c r="I47" s="8">
+      <c r="I47">
         <v>5</v>
       </c>
-      <c r="J47" s="8">
+      <c r="J47">
         <v>9</v>
       </c>
-      <c r="K47" s="8">
+      <c r="K47">
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="8">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A48">
         <v>52</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B48" t="s">
         <v>110</v>
       </c>
-      <c r="C48" s="8">
+      <c r="C48">
         <v>46</v>
       </c>
-      <c r="D48" s="8" t="s">
+      <c r="D48" t="s">
         <v>110</v>
       </c>
-      <c r="E48" s="8">
+      <c r="E48">
         <v>0.2</v>
       </c>
-      <c r="F48" s="8">
+      <c r="F48">
         <v>0</v>
       </c>
-      <c r="G48" s="8">
+      <c r="G48">
         <v>9.4</v>
       </c>
-      <c r="H48" s="8">
+      <c r="H48">
         <v>0</v>
       </c>
-      <c r="I48" s="8">
-        <v>3</v>
-      </c>
-      <c r="J48" s="8">
+      <c r="I48">
+        <v>3</v>
+      </c>
+      <c r="J48">
         <v>11</v>
       </c>
-      <c r="K48" s="8">
+      <c r="K48">
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="8">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A49">
         <v>53</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" t="s">
         <v>111</v>
       </c>
-      <c r="C49" s="8">
+      <c r="C49">
         <v>125</v>
       </c>
-      <c r="D49" s="8" t="s">
+      <c r="D49" t="s">
         <v>111</v>
       </c>
-      <c r="E49" s="8">
-        <v>3</v>
-      </c>
-      <c r="F49" s="8">
+      <c r="E49">
+        <v>3</v>
+      </c>
+      <c r="F49">
         <v>0.05</v>
       </c>
-      <c r="G49" s="8">
+      <c r="G49">
         <v>0</v>
       </c>
-      <c r="H49" s="8">
+      <c r="H49">
         <v>0.5</v>
       </c>
-      <c r="I49" s="8">
+      <c r="I49">
         <v>2</v>
       </c>
-      <c r="J49" s="8">
+      <c r="J49">
         <v>8</v>
       </c>
-      <c r="K49" s="8">
+      <c r="K49">
         <v>30</v>
       </c>
     </row>
-    <row r="50" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="8">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A50">
         <v>56</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" t="s">
         <v>112</v>
       </c>
-      <c r="C50" s="8">
+      <c r="C50">
         <v>64</v>
       </c>
-      <c r="D50" s="8" t="s">
+      <c r="D50" t="s">
         <v>112</v>
       </c>
-      <c r="E50" s="8">
+      <c r="E50">
         <v>0</v>
       </c>
-      <c r="F50" s="8">
+      <c r="F50">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="G50" s="8">
+      <c r="G50">
         <v>17</v>
       </c>
-      <c r="H50" s="8">
+      <c r="H50">
         <v>0</v>
       </c>
-      <c r="I50" s="8">
+      <c r="I50">
         <v>5</v>
       </c>
-      <c r="J50" s="8">
+      <c r="J50">
         <v>16</v>
       </c>
-      <c r="K50" s="8">
+      <c r="K50">
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="8">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A51">
         <v>57</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B51" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="8">
+      <c r="C51">
         <v>74</v>
       </c>
-      <c r="D51" s="8" t="s">
+      <c r="D51" t="s">
         <v>113</v>
       </c>
-      <c r="E51" s="8">
+      <c r="E51">
         <v>0.2</v>
       </c>
-      <c r="F51" s="8">
+      <c r="F51">
         <v>0.01</v>
       </c>
-      <c r="G51" s="8">
+      <c r="G51">
         <v>16</v>
       </c>
-      <c r="H51" s="8">
+      <c r="H51">
         <v>0.1</v>
       </c>
-      <c r="I51" s="8">
-        <v>3</v>
-      </c>
-      <c r="J51" s="8">
-        <v>3</v>
-      </c>
-      <c r="K51" s="8">
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="8">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A52">
         <v>58</v>
       </c>
-      <c r="B52" s="8" t="s">
+      <c r="B52" t="s">
         <v>114</v>
       </c>
-      <c r="C52" s="8">
+      <c r="C52">
         <v>14</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="D52" t="s">
         <v>114</v>
       </c>
-      <c r="E52" s="8">
+      <c r="E52">
         <v>0.1</v>
       </c>
-      <c r="F52" s="8">
+      <c r="F52">
         <v>0.02</v>
       </c>
-      <c r="G52" s="8">
+      <c r="G52">
         <v>1.5</v>
       </c>
-      <c r="H52" s="8">
+      <c r="H52">
         <v>0.04</v>
       </c>
-      <c r="I52" s="8">
-        <v>3</v>
-      </c>
-      <c r="J52" s="8">
+      <c r="I52">
+        <v>3</v>
+      </c>
+      <c r="J52">
         <v>8</v>
       </c>
-      <c r="K52" s="8">
+      <c r="K52">
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="8">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A53">
         <v>59</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" t="s">
         <v>115</v>
       </c>
-      <c r="C53" s="8">
+      <c r="C53">
         <v>45</v>
       </c>
-      <c r="D53" s="8" t="s">
+      <c r="D53" t="s">
         <v>115</v>
       </c>
-      <c r="E53" s="8">
+      <c r="E53">
         <v>0.2</v>
       </c>
-      <c r="F53" s="8">
+      <c r="F53">
         <v>0.01</v>
       </c>
-      <c r="G53" s="8">
+      <c r="G53">
         <v>7</v>
       </c>
-      <c r="H53" s="8">
+      <c r="H53">
         <v>0.01</v>
       </c>
-      <c r="I53" s="8">
+      <c r="I53">
         <v>2</v>
       </c>
-      <c r="J53" s="8">
+      <c r="J53">
         <v>16</v>
       </c>
-      <c r="K53" s="8">
+      <c r="K53">
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="8">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A54">
         <v>60</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" t="s">
         <v>116</v>
       </c>
-      <c r="C54" s="8">
+      <c r="C54">
         <v>60</v>
       </c>
-      <c r="D54" s="8" t="s">
+      <c r="D54" t="s">
         <v>116</v>
       </c>
-      <c r="E54" s="8">
+      <c r="E54">
         <v>0.2</v>
       </c>
-      <c r="F54" s="8">
+      <c r="F54">
         <v>0.02</v>
       </c>
-      <c r="G54" s="8">
+      <c r="G54">
         <v>14</v>
       </c>
-      <c r="H54" s="8">
+      <c r="H54">
         <v>0</v>
       </c>
-      <c r="I54" s="8">
-        <v>3</v>
-      </c>
-      <c r="J54" s="8">
+      <c r="I54">
+        <v>3</v>
+      </c>
+      <c r="J54">
         <v>9</v>
       </c>
-      <c r="K54" s="8">
+      <c r="K54">
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="8">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A55">
         <v>61</v>
       </c>
-      <c r="B55" s="8" t="s">
+      <c r="B55" t="s">
         <v>117</v>
       </c>
-      <c r="C55" s="8">
+      <c r="C55">
         <v>64</v>
       </c>
-      <c r="D55" s="8" t="s">
+      <c r="D55" t="s">
         <v>117</v>
       </c>
-      <c r="E55" s="8">
+      <c r="E55">
         <v>0.4</v>
       </c>
-      <c r="F55" s="8">
+      <c r="F55">
         <v>0</v>
       </c>
-      <c r="G55" s="8">
+      <c r="G55">
         <v>5</v>
       </c>
-      <c r="H55" s="8">
+      <c r="H55">
         <v>0.02</v>
       </c>
-      <c r="I55" s="8">
+      <c r="I55">
         <v>2</v>
       </c>
-      <c r="J55" s="8">
+      <c r="J55">
         <v>10</v>
       </c>
-      <c r="K55" s="8">
+      <c r="K55">
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="8">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A56">
         <v>62</v>
       </c>
-      <c r="B56" s="8" t="s">
+      <c r="B56" t="s">
         <v>118</v>
       </c>
-      <c r="C56" s="8">
+      <c r="C56">
         <v>25</v>
       </c>
-      <c r="D56" s="8" t="s">
+      <c r="D56" t="s">
         <v>118</v>
       </c>
-      <c r="E56" s="8">
+      <c r="E56">
         <v>0.7</v>
       </c>
-      <c r="F56" s="8">
+      <c r="F56">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G56" s="8">
+      <c r="G56">
         <v>0.35</v>
       </c>
-      <c r="H56" s="8">
+      <c r="H56">
         <v>0.08</v>
       </c>
-      <c r="I56" s="8">
+      <c r="I56">
         <v>2</v>
       </c>
-      <c r="J56" s="8">
+      <c r="J56">
         <v>10</v>
       </c>
-      <c r="K56" s="8">
+      <c r="K56">
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="8">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A57">
         <v>63</v>
       </c>
-      <c r="B57" s="8" t="s">
+      <c r="B57" t="s">
         <v>119</v>
       </c>
-      <c r="C57" s="8">
+      <c r="C57">
         <v>35</v>
       </c>
-      <c r="D57" s="8" t="s">
+      <c r="D57" t="s">
         <v>119</v>
       </c>
-      <c r="E57" s="8">
+      <c r="E57">
         <v>0.2</v>
       </c>
-      <c r="F57" s="8">
+      <c r="F57">
         <v>0</v>
       </c>
-      <c r="G57" s="8">
+      <c r="G57">
         <v>6.5</v>
       </c>
-      <c r="H57" s="8">
+      <c r="H57">
         <v>0</v>
       </c>
-      <c r="I57" s="8">
-        <v>3</v>
-      </c>
-      <c r="J57" s="8">
-        <v>3</v>
-      </c>
-      <c r="K57" s="8">
+      <c r="I57">
+        <v>3</v>
+      </c>
+      <c r="J57">
+        <v>3</v>
+      </c>
+      <c r="K57">
         <v>15</v>
       </c>
     </row>
-    <row r="58" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="8">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A58">
         <v>64</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="B58" t="s">
         <v>120</v>
       </c>
-      <c r="C58" s="8">
+      <c r="C58">
         <v>22</v>
       </c>
-      <c r="D58" s="8" t="s">
+      <c r="D58" t="s">
         <v>120</v>
       </c>
-      <c r="E58" s="8">
+      <c r="E58">
         <v>0.1</v>
       </c>
-      <c r="F58" s="8">
+      <c r="F58">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="G58" s="8">
+      <c r="G58">
         <v>2.8</v>
       </c>
-      <c r="H58" s="8">
+      <c r="H58">
         <v>0.05</v>
       </c>
-      <c r="I58" s="8">
-        <v>3</v>
-      </c>
-      <c r="J58" s="8">
+      <c r="I58">
+        <v>3</v>
+      </c>
+      <c r="J58">
         <v>9</v>
       </c>
-      <c r="K58" s="8">
+      <c r="K58">
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="8">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A59">
         <v>65</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B59" t="s">
         <v>121</v>
       </c>
-      <c r="C59" s="8">
+      <c r="C59">
         <v>30</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D59" t="s">
         <v>121</v>
       </c>
-      <c r="E59" s="8">
+      <c r="E59">
         <v>0.2</v>
       </c>
-      <c r="F59" s="8">
+      <c r="F59">
         <v>0.02</v>
       </c>
-      <c r="G59" s="8">
+      <c r="G59">
         <v>5.0999999999999996</v>
       </c>
-      <c r="H59" s="8">
+      <c r="H59">
         <v>0.1</v>
       </c>
-      <c r="I59" s="8">
-        <v>3</v>
-      </c>
-      <c r="J59" s="8">
+      <c r="I59">
+        <v>3</v>
+      </c>
+      <c r="J59">
         <v>16</v>
       </c>
-      <c r="K59" s="8">
+      <c r="K59">
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="8">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A60">
         <v>66</v>
       </c>
-      <c r="B60" s="8" t="s">
+      <c r="B60" t="s">
         <v>122</v>
       </c>
-      <c r="C60" s="8">
+      <c r="C60">
         <v>25</v>
       </c>
-      <c r="D60" s="8" t="s">
+      <c r="D60" t="s">
         <v>122</v>
       </c>
-      <c r="E60" s="8">
+      <c r="E60">
         <v>0</v>
       </c>
-      <c r="F60" s="8">
+      <c r="F60">
         <v>0.02</v>
       </c>
-      <c r="G60" s="8">
+      <c r="G60">
         <v>5</v>
       </c>
-      <c r="H60" s="8">
+      <c r="H60">
         <v>0</v>
       </c>
-      <c r="I60" s="8">
+      <c r="I60">
         <v>2</v>
       </c>
-      <c r="J60" s="8">
+      <c r="J60">
         <v>11</v>
       </c>
-      <c r="K60" s="8">
+      <c r="K60">
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="8">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A61">
         <v>67</v>
       </c>
-      <c r="B61" s="8" t="s">
+      <c r="B61" t="s">
+        <v>132</v>
+      </c>
+      <c r="C61">
+        <v>87</v>
+      </c>
+      <c r="D61" t="s">
+        <v>132</v>
+      </c>
+      <c r="E61">
+        <v>0.3</v>
+      </c>
+      <c r="F61">
+        <v>0.03</v>
+      </c>
+      <c r="G61">
+        <v>18</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61">
+        <v>2</v>
+      </c>
+      <c r="J61">
+        <v>9</v>
+      </c>
+      <c r="K61">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>69</v>
+      </c>
+      <c r="B62" t="s">
         <v>133</v>
       </c>
-      <c r="C61" s="8">
-        <v>87</v>
-      </c>
-      <c r="D61" s="8" t="s">
+      <c r="C62">
+        <v>125</v>
+      </c>
+      <c r="D62" t="s">
         <v>133</v>
       </c>
-      <c r="E61" s="8">
+      <c r="E62">
+        <v>0.2</v>
+      </c>
+      <c r="F62">
+        <v>0.03</v>
+      </c>
+      <c r="G62">
+        <v>3</v>
+      </c>
+      <c r="H62">
+        <v>0.1</v>
+      </c>
+      <c r="I62">
+        <v>5</v>
+      </c>
+      <c r="J62">
+        <v>2</v>
+      </c>
+      <c r="K62">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>71</v>
+      </c>
+      <c r="B63" t="s">
+        <v>134</v>
+      </c>
+      <c r="C63">
+        <v>30</v>
+      </c>
+      <c r="D63" t="s">
+        <v>134</v>
+      </c>
+      <c r="E63">
+        <v>0.2</v>
+      </c>
+      <c r="F63">
+        <v>0.01</v>
+      </c>
+      <c r="G63">
+        <v>3</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <v>3</v>
+      </c>
+      <c r="J63">
+        <v>8</v>
+      </c>
+      <c r="K63">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>72</v>
+      </c>
+      <c r="B64" t="s">
+        <v>135</v>
+      </c>
+      <c r="C64">
+        <v>19</v>
+      </c>
+      <c r="D64" t="s">
+        <v>135</v>
+      </c>
+      <c r="E64">
+        <v>0.1</v>
+      </c>
+      <c r="F64">
+        <v>0.02</v>
+      </c>
+      <c r="G64">
+        <v>1</v>
+      </c>
+      <c r="H64">
+        <v>0.01</v>
+      </c>
+      <c r="I64">
+        <v>2</v>
+      </c>
+      <c r="J64">
+        <v>16</v>
+      </c>
+      <c r="K64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>73</v>
+      </c>
+      <c r="B65" t="s">
+        <v>136</v>
+      </c>
+      <c r="C65">
+        <v>38</v>
+      </c>
+      <c r="D65" t="s">
+        <v>137</v>
+      </c>
+      <c r="E65">
+        <v>0.6</v>
+      </c>
+      <c r="F65">
+        <v>0.02</v>
+      </c>
+      <c r="G65">
+        <v>2</v>
+      </c>
+      <c r="H65">
+        <v>0.05</v>
+      </c>
+      <c r="I65">
+        <v>2</v>
+      </c>
+      <c r="J65">
+        <v>10</v>
+      </c>
+      <c r="K65">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>75</v>
+      </c>
+      <c r="B66" t="s">
+        <v>138</v>
+      </c>
+      <c r="C66">
+        <v>200</v>
+      </c>
+      <c r="D66" t="s">
+        <v>138</v>
+      </c>
+      <c r="E66">
+        <v>8</v>
+      </c>
+      <c r="F66">
+        <v>1.5</v>
+      </c>
+      <c r="G66">
+        <v>3</v>
+      </c>
+      <c r="H66">
+        <v>3.5</v>
+      </c>
+      <c r="I66">
+        <v>2</v>
+      </c>
+      <c r="J66">
+        <v>2</v>
+      </c>
+      <c r="K66">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>76</v>
+      </c>
+      <c r="B67" t="s">
+        <v>139</v>
+      </c>
+      <c r="C67">
+        <v>312</v>
+      </c>
+      <c r="D67" t="s">
+        <v>140</v>
+      </c>
+      <c r="E67">
+        <v>12</v>
+      </c>
+      <c r="F67">
+        <v>0.03</v>
+      </c>
+      <c r="G67">
+        <v>1.3</v>
+      </c>
+      <c r="H67">
+        <v>3</v>
+      </c>
+      <c r="I67">
+        <v>2</v>
+      </c>
+      <c r="J67">
+        <v>2</v>
+      </c>
+      <c r="K67">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>77</v>
+      </c>
+      <c r="B68" t="s">
+        <v>141</v>
+      </c>
+      <c r="C68">
+        <v>140</v>
+      </c>
+      <c r="D68" t="s">
+        <v>141</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>35</v>
+      </c>
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68">
+        <v>5</v>
+      </c>
+      <c r="J68">
+        <v>2</v>
+      </c>
+      <c r="K68">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>79</v>
+      </c>
+      <c r="B69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C69">
+        <v>135</v>
+      </c>
+      <c r="D69" t="s">
+        <v>143</v>
+      </c>
+      <c r="E69">
+        <v>3</v>
+      </c>
+      <c r="F69">
+        <v>0.1</v>
+      </c>
+      <c r="G69">
+        <v>12</v>
+      </c>
+      <c r="H69">
+        <v>4</v>
+      </c>
+      <c r="I69">
+        <v>2</v>
+      </c>
+      <c r="J69">
+        <v>2</v>
+      </c>
+      <c r="K69">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>80</v>
+      </c>
+      <c r="B70" t="s">
+        <v>144</v>
+      </c>
+      <c r="C70">
+        <v>90</v>
+      </c>
+      <c r="D70" t="s">
+        <v>144</v>
+      </c>
+      <c r="E70">
+        <v>1</v>
+      </c>
+      <c r="F70">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="G70">
+        <v>0</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
+        <v>4</v>
+      </c>
+      <c r="J70">
+        <v>10</v>
+      </c>
+      <c r="K70">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>81</v>
+      </c>
+      <c r="B71" t="s">
+        <v>145</v>
+      </c>
+      <c r="C71">
+        <v>80</v>
+      </c>
+      <c r="D71" t="s">
+        <v>145</v>
+      </c>
+      <c r="E71">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F71">
+        <v>0.05</v>
+      </c>
+      <c r="G71">
+        <v>0</v>
+      </c>
+      <c r="H71">
+        <v>0</v>
+      </c>
+      <c r="I71">
+        <v>3</v>
+      </c>
+      <c r="J71">
+        <v>10</v>
+      </c>
+      <c r="K71">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>82</v>
+      </c>
+      <c r="B72" t="s">
+        <v>146</v>
+      </c>
+      <c r="C72">
+        <v>250</v>
+      </c>
+      <c r="D72" t="s">
+        <v>146</v>
+      </c>
+      <c r="E72">
+        <v>8</v>
+      </c>
+      <c r="F72">
         <v>0.3</v>
       </c>
-      <c r="F61" s="8">
-        <v>0.03</v>
-      </c>
-      <c r="G61" s="8">
-        <v>18</v>
-      </c>
-      <c r="H61" s="8">
-        <v>0</v>
-      </c>
-      <c r="I61" s="8">
+      <c r="G72">
+        <v>5</v>
+      </c>
+      <c r="H72">
+        <v>3</v>
+      </c>
+      <c r="I72">
         <v>2</v>
       </c>
-      <c r="J61" s="8">
-        <v>9</v>
-      </c>
-      <c r="K61" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="8">
-        <v>69</v>
-      </c>
-      <c r="B62" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="C62" s="8">
-        <v>125</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="E62" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="F62" s="8">
-        <v>0.03</v>
-      </c>
-      <c r="G62" s="8">
-        <v>3</v>
-      </c>
-      <c r="H62" s="8">
-        <v>0.1</v>
-      </c>
-      <c r="I62" s="8">
-        <v>5</v>
-      </c>
-      <c r="J62" s="8">
-        <v>2</v>
-      </c>
-      <c r="K62" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="8">
-        <v>71</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="C63" s="8">
-        <v>30</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="E63" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="F63" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="G63" s="8">
-        <v>3</v>
-      </c>
-      <c r="H63" s="8">
-        <v>0</v>
-      </c>
-      <c r="I63" s="8">
-        <v>3</v>
-      </c>
-      <c r="J63" s="8">
+      <c r="J72">
         <v>8</v>
       </c>
-      <c r="K63" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="8">
-        <v>72</v>
-      </c>
-      <c r="B64" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="C64" s="8">
-        <v>19</v>
-      </c>
-      <c r="D64" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="E64" s="8">
-        <v>0.1</v>
-      </c>
-      <c r="F64" s="8">
-        <v>0.02</v>
-      </c>
-      <c r="G64" s="8">
-        <v>1</v>
-      </c>
-      <c r="H64" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="I64" s="8">
-        <v>2</v>
-      </c>
-      <c r="J64" s="8">
-        <v>16</v>
-      </c>
-      <c r="K64" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="8">
-        <v>73</v>
-      </c>
-      <c r="B65" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C65" s="8">
-        <v>38</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="E65" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="F65" s="8">
-        <v>0.02</v>
-      </c>
-      <c r="G65" s="8">
-        <v>2</v>
-      </c>
-      <c r="H65" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="I65" s="8">
-        <v>2</v>
-      </c>
-      <c r="J65" s="8">
-        <v>10</v>
-      </c>
-      <c r="K65" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="66" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="8">
-        <v>75</v>
-      </c>
-      <c r="B66" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="C66" s="8">
-        <v>200</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="E66" s="8">
-        <v>8</v>
-      </c>
-      <c r="F66" s="8">
-        <v>1.5</v>
-      </c>
-      <c r="G66" s="8">
-        <v>3</v>
-      </c>
-      <c r="H66" s="8">
-        <v>3.5</v>
-      </c>
-      <c r="I66" s="8">
-        <v>2</v>
-      </c>
-      <c r="J66" s="8">
-        <v>2</v>
-      </c>
-      <c r="K66" s="8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="67" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="8">
-        <v>76</v>
-      </c>
-      <c r="B67" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C67" s="8">
-        <v>312</v>
-      </c>
-      <c r="D67" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="E67" s="8">
-        <v>12</v>
-      </c>
-      <c r="F67" s="8">
-        <v>0.03</v>
-      </c>
-      <c r="G67" s="8">
-        <v>1.3</v>
-      </c>
-      <c r="H67" s="8">
-        <v>3</v>
-      </c>
-      <c r="I67" s="8">
-        <v>2</v>
-      </c>
-      <c r="J67" s="8">
-        <v>2</v>
-      </c>
-      <c r="K67" s="8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="8">
-        <v>77</v>
-      </c>
-      <c r="B68" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="C68" s="8">
-        <v>140</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="E68" s="8">
-        <v>0</v>
-      </c>
-      <c r="F68" s="8">
-        <v>0</v>
-      </c>
-      <c r="G68" s="8">
-        <v>35</v>
-      </c>
-      <c r="H68" s="8">
-        <v>0</v>
-      </c>
-      <c r="I68" s="8">
-        <v>5</v>
-      </c>
-      <c r="J68" s="8">
-        <v>2</v>
-      </c>
-      <c r="K68" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="69" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="8">
-        <v>79</v>
-      </c>
-      <c r="B69" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="C69" s="8">
-        <v>135</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="E69" s="8">
-        <v>3</v>
-      </c>
-      <c r="F69" s="8">
-        <v>0.1</v>
-      </c>
-      <c r="G69" s="8">
-        <v>12</v>
-      </c>
-      <c r="H69" s="8">
-        <v>4</v>
-      </c>
-      <c r="I69" s="8">
-        <v>2</v>
-      </c>
-      <c r="J69" s="8">
-        <v>2</v>
-      </c>
-      <c r="K69" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="70" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="8">
-        <v>80</v>
-      </c>
-      <c r="B70" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="C70" s="8">
-        <v>90</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="E70" s="8">
-        <v>1</v>
-      </c>
-      <c r="F70" s="8">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="G70" s="8">
-        <v>0</v>
-      </c>
-      <c r="H70" s="8">
-        <v>0</v>
-      </c>
-      <c r="I70" s="8">
-        <v>4</v>
-      </c>
-      <c r="J70" s="8">
-        <v>10</v>
-      </c>
-      <c r="K70" s="8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="71" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="8">
-        <v>81</v>
-      </c>
-      <c r="B71" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="C71" s="8">
-        <v>80</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="E71" s="8">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F71" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="G71" s="8">
-        <v>0</v>
-      </c>
-      <c r="H71" s="8">
-        <v>0</v>
-      </c>
-      <c r="I71" s="8">
-        <v>3</v>
-      </c>
-      <c r="J71" s="8">
-        <v>10</v>
-      </c>
-      <c r="K71" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="72" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="8">
-        <v>82</v>
-      </c>
-      <c r="B72" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C72" s="8">
-        <v>250</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="E72" s="8">
-        <v>8</v>
-      </c>
-      <c r="F72" s="8">
-        <v>0.3</v>
-      </c>
-      <c r="G72" s="8">
-        <v>5</v>
-      </c>
-      <c r="H72" s="8">
-        <v>3</v>
-      </c>
-      <c r="I72" s="8">
-        <v>2</v>
-      </c>
-      <c r="J72" s="8">
-        <v>8</v>
-      </c>
-      <c r="K72" s="8">
+      <c r="K72">
         <v>30</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.35">
       <c r="I75" t="s">
+        <v>152</v>
+      </c>
+      <c r="J75" t="s">
+        <v>148</v>
+      </c>
+      <c r="K75" t="s">
+        <v>149</v>
+      </c>
+      <c r="L75" t="s">
+        <v>150</v>
+      </c>
+      <c r="M75" t="s">
         <v>153</v>
       </c>
-      <c r="J75" t="s">
-        <v>149</v>
-      </c>
-      <c r="K75" t="s">
-        <v>150</v>
-      </c>
-      <c r="L75" t="s">
-        <v>151</v>
-      </c>
-      <c r="M75" t="s">
+      <c r="N75" t="s">
         <v>154</v>
       </c>
-      <c r="N75" t="s">
-        <v>155</v>
-      </c>
       <c r="O75" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.35">
@@ -4158,21 +4157,21 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5" t="s">
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5" t="s">
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
@@ -4226,10 +4225,10 @@
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C15" t="s">
@@ -4279,8 +4278,8 @@
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A16" s="4"/>
-      <c r="B16" s="7"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="5"/>
       <c r="C16" t="s">
         <v>66</v>
       </c>
@@ -4328,8 +4327,8 @@
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A17" s="4"/>
-      <c r="B17" s="7"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="5"/>
       <c r="C17" t="s">
         <v>67</v>
       </c>
@@ -4352,7 +4351,7 @@
         <v>72</v>
       </c>
       <c r="K17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L17">
         <v>19</v>
@@ -4370,17 +4369,17 @@
         <v>80</v>
       </c>
       <c r="Q17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="R17">
         <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>68</v>
       </c>
       <c r="C18" t="s">
@@ -4430,8 +4429,8 @@
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A19" s="4"/>
-      <c r="B19" s="7"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="5"/>
       <c r="C19" t="s">
         <v>70</v>
       </c>
@@ -4479,8 +4478,8 @@
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A20" s="4"/>
-      <c r="B20" s="7"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="5"/>
       <c r="C20" t="s">
         <v>71</v>
       </c>
@@ -4528,10 +4527,10 @@
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="5" t="s">
         <v>72</v>
       </c>
       <c r="C21" t="s">
@@ -4581,8 +4580,8 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A22" s="4"/>
-      <c r="B22" s="7"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="5"/>
       <c r="C22" t="s">
         <v>74</v>
       </c>
@@ -4605,7 +4604,7 @@
         <v>71</v>
       </c>
       <c r="K22" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="L22">
         <v>30</v>
@@ -4630,8 +4629,8 @@
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A23" s="4"/>
-      <c r="B23" s="7"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="5"/>
       <c r="C23" t="s">
         <v>75</v>
       </c>
@@ -4679,10 +4678,10 @@
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="B24" s="7" t="s">
+      <c r="A24" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C24" t="s">
@@ -4725,15 +4724,15 @@
         <v>69</v>
       </c>
       <c r="Q24" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="R24">
         <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A25" s="4"/>
-      <c r="B25" s="7"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="5"/>
       <c r="C25" t="s">
         <v>78</v>
       </c>
@@ -4781,8 +4780,8 @@
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A26" s="4"/>
-      <c r="B26" s="7"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="5"/>
       <c r="C26" t="s">
         <v>79</v>
       </c>
@@ -4805,7 +4804,7 @@
         <v>73</v>
       </c>
       <c r="K26" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L26">
         <v>38</v>
@@ -4830,10 +4829,10 @@
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B27" s="7" t="s">
+      <c r="A27" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C27" t="s">
@@ -4883,8 +4882,8 @@
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A28" s="4"/>
-      <c r="B28" s="7"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="5"/>
       <c r="C28" t="s">
         <v>82</v>
       </c>
@@ -4925,15 +4924,15 @@
         <v>79</v>
       </c>
       <c r="Q28" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="R28">
         <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A29" s="4"/>
-      <c r="B29" s="7"/>
+      <c r="A29" s="7"/>
+      <c r="B29" s="5"/>
       <c r="C29" t="s">
         <v>83</v>
       </c>
@@ -4974,17 +4973,17 @@
         <v>77</v>
       </c>
       <c r="Q29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="R29">
         <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="5" t="s">
         <v>84</v>
       </c>
       <c r="C30" t="s">
@@ -5018,7 +5017,7 @@
         <v>81</v>
       </c>
       <c r="N30" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O30">
         <v>80</v>
@@ -5034,8 +5033,8 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A31" s="4"/>
-      <c r="B31" s="7"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="5"/>
       <c r="C31" t="s">
         <v>86</v>
       </c>
@@ -5083,8 +5082,8 @@
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A32" s="4"/>
-      <c r="B32" s="7"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="5"/>
       <c r="C32" t="s">
         <v>87</v>
       </c>
@@ -5116,7 +5115,7 @@
         <v>67</v>
       </c>
       <c r="N32" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O32">
         <v>87</v>
@@ -5132,10 +5131,10 @@
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A33" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="B33" s="6" t="s">
+      <c r="A33" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C33" t="s">
@@ -5185,8 +5184,8 @@
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A34" s="4"/>
-      <c r="B34" s="6"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="4"/>
       <c r="C34" t="s">
         <v>90</v>
       </c>
@@ -5234,8 +5233,8 @@
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A35" s="4"/>
-      <c r="B35" s="6"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="4"/>
       <c r="C35" t="s">
         <v>91</v>
       </c>
@@ -5267,7 +5266,7 @@
         <v>80</v>
       </c>
       <c r="N35" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O35">
         <v>90</v>
@@ -5283,10 +5282,10 @@
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A36" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="B36" s="7" t="s">
+      <c r="A36" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>92</v>
       </c>
       <c r="C36" t="s">
@@ -5336,8 +5335,8 @@
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A37" s="4"/>
-      <c r="B37" s="7"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="5"/>
       <c r="C37" t="s">
         <v>94</v>
       </c>
@@ -5378,15 +5377,15 @@
         <v>75</v>
       </c>
       <c r="Q37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="R37">
         <v>200</v>
       </c>
     </row>
     <row r="38" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="4"/>
-      <c r="B38" s="7"/>
+      <c r="A38" s="7"/>
+      <c r="B38" s="5"/>
       <c r="C38" s="3" t="s">
         <v>95</v>
       </c>
@@ -5434,10 +5433,10 @@
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="5" t="s">
         <v>96</v>
       </c>
       <c r="C39" t="s">
@@ -5487,8 +5486,8 @@
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A40" s="4"/>
-      <c r="B40" s="7"/>
+      <c r="A40" s="7"/>
+      <c r="B40" s="5"/>
       <c r="C40" t="s">
         <v>98</v>
       </c>
@@ -5536,8 +5535,8 @@
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A41" s="4"/>
-      <c r="B41" s="7"/>
+      <c r="A41" s="7"/>
+      <c r="B41" s="5"/>
       <c r="C41" t="s">
         <v>99</v>
       </c>
@@ -5578,17 +5577,17 @@
         <v>82</v>
       </c>
       <c r="Q41" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="R41">
         <v>250</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A42" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B42" s="7" t="s">
+      <c r="A42" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>100</v>
       </c>
       <c r="C42" t="s">
@@ -5622,7 +5621,7 @@
         <v>69</v>
       </c>
       <c r="N42" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O42">
         <v>125</v>
@@ -5638,8 +5637,8 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A43" s="4"/>
-      <c r="B43" s="7"/>
+      <c r="A43" s="7"/>
+      <c r="B43" s="5"/>
       <c r="C43" t="s">
         <v>102</v>
       </c>
@@ -5662,7 +5661,7 @@
         <v>81</v>
       </c>
       <c r="K43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L43">
         <v>80</v>
@@ -5687,8 +5686,8 @@
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A44" s="4"/>
-      <c r="B44" s="7"/>
+      <c r="A44" s="7"/>
+      <c r="B44" s="5"/>
       <c r="C44" t="s">
         <v>103</v>
       </c>
@@ -5729,7 +5728,7 @@
         <v>76</v>
       </c>
       <c r="Q44" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="R44">
         <v>312</v>
@@ -5737,6 +5736,19 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A20"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="B39:B41"/>
@@ -5747,19 +5759,6 @@
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B30:B32"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="P13:R13"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A36:A38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated tutorial and added fridge mechanic
</commit_message>
<xml_diff>
--- a/Food Progression.xlsx
+++ b/Food Progression.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Nutri Mayhem\NutriCrush-Unity-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA98762-EE3C-498C-9527-17FE9498C110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE15FB26-A830-4388-8230-F36FDDA13DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8110" yWindow="3210" windowWidth="21600" windowHeight="14680" activeTab="1" xr2:uid="{3A71858E-782A-488A-BF56-898FF2A6D53B}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{3A71858E-782A-488A-BF56-898FF2A6D53B}"/>
   </bookViews>
   <sheets>
     <sheet name="Food" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="156">
   <si>
     <t>Id</t>
   </si>
@@ -1001,16 +1001,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4099,6 +4099,15 @@
       <c r="E8">
         <v>3</v>
       </c>
+      <c r="J8">
+        <v>30</v>
+      </c>
+      <c r="K8" t="s">
+        <v>42</v>
+      </c>
+      <c r="L8">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9">
@@ -4116,13 +4125,13 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="D10">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -4157,21 +4166,21 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6" t="s">
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6" t="s">
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
@@ -4225,10 +4234,10 @@
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="7" t="s">
         <v>64</v>
       </c>
       <c r="C15" t="s">
@@ -4259,13 +4268,13 @@
         <v>14</v>
       </c>
       <c r="M15">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="N15" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="O15">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="P15">
         <v>22</v>
@@ -4278,8 +4287,8 @@
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A16" s="7"/>
-      <c r="B16" s="5"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="7"/>
       <c r="C16" t="s">
         <v>66</v>
       </c>
@@ -4308,13 +4317,13 @@
         <v>17</v>
       </c>
       <c r="M16">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="N16" t="s">
-        <v>115</v>
+        <v>46</v>
       </c>
       <c r="O16">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="P16">
         <v>51</v>
@@ -4327,8 +4336,8 @@
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A17" s="7"/>
-      <c r="B17" s="5"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="7"/>
       <c r="C17" t="s">
         <v>67</v>
       </c>
@@ -4357,10 +4366,10 @@
         <v>19</v>
       </c>
       <c r="M17">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="N17" t="s">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="O17">
         <v>45</v>
@@ -4376,10 +4385,10 @@
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>68</v>
       </c>
       <c r="C18" t="s">
@@ -4429,8 +4438,8 @@
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A19" s="7"/>
-      <c r="B19" s="5"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="7"/>
       <c r="C19" t="s">
         <v>70</v>
       </c>
@@ -4478,8 +4487,8 @@
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A20" s="7"/>
-      <c r="B20" s="5"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="7"/>
       <c r="C20" t="s">
         <v>71</v>
       </c>
@@ -4527,10 +4536,10 @@
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="7" t="s">
         <v>72</v>
       </c>
       <c r="C21" t="s">
@@ -4580,8 +4589,8 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A22" s="7"/>
-      <c r="B22" s="5"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="7"/>
       <c r="C22" t="s">
         <v>74</v>
       </c>
@@ -4629,8 +4638,8 @@
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A23" s="7"/>
-      <c r="B23" s="5"/>
+      <c r="A23" s="4"/>
+      <c r="B23" s="7"/>
       <c r="C23" t="s">
         <v>75</v>
       </c>
@@ -4678,10 +4687,10 @@
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="7" t="s">
         <v>76</v>
       </c>
       <c r="C24" t="s">
@@ -4731,8 +4740,8 @@
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A25" s="7"/>
-      <c r="B25" s="5"/>
+      <c r="A25" s="4"/>
+      <c r="B25" s="7"/>
       <c r="C25" t="s">
         <v>78</v>
       </c>
@@ -4780,8 +4789,8 @@
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A26" s="7"/>
-      <c r="B26" s="5"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="7"/>
       <c r="C26" t="s">
         <v>79</v>
       </c>
@@ -4829,10 +4838,10 @@
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
         <v>80</v>
       </c>
       <c r="C27" t="s">
@@ -4882,8 +4891,8 @@
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A28" s="7"/>
-      <c r="B28" s="5"/>
+      <c r="A28" s="4"/>
+      <c r="B28" s="7"/>
       <c r="C28" t="s">
         <v>82</v>
       </c>
@@ -4931,8 +4940,8 @@
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A29" s="7"/>
-      <c r="B29" s="5"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="7"/>
       <c r="C29" t="s">
         <v>83</v>
       </c>
@@ -4980,10 +4989,10 @@
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="7" t="s">
         <v>84</v>
       </c>
       <c r="C30" t="s">
@@ -5033,8 +5042,8 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A31" s="7"/>
-      <c r="B31" s="5"/>
+      <c r="A31" s="4"/>
+      <c r="B31" s="7"/>
       <c r="C31" t="s">
         <v>86</v>
       </c>
@@ -5082,8 +5091,8 @@
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A32" s="7"/>
-      <c r="B32" s="5"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="7"/>
       <c r="C32" t="s">
         <v>87</v>
       </c>
@@ -5131,10 +5140,10 @@
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="6" t="s">
         <v>88</v>
       </c>
       <c r="C33" t="s">
@@ -5184,8 +5193,8 @@
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A34" s="7"/>
-      <c r="B34" s="4"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="6"/>
       <c r="C34" t="s">
         <v>90</v>
       </c>
@@ -5233,8 +5242,8 @@
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A35" s="7"/>
-      <c r="B35" s="4"/>
+      <c r="A35" s="4"/>
+      <c r="B35" s="6"/>
       <c r="C35" t="s">
         <v>91</v>
       </c>
@@ -5282,10 +5291,10 @@
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="7" t="s">
         <v>92</v>
       </c>
       <c r="C36" t="s">
@@ -5335,8 +5344,8 @@
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A37" s="7"/>
-      <c r="B37" s="5"/>
+      <c r="A37" s="4"/>
+      <c r="B37" s="7"/>
       <c r="C37" t="s">
         <v>94</v>
       </c>
@@ -5384,8 +5393,8 @@
       </c>
     </row>
     <row r="38" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="7"/>
-      <c r="B38" s="5"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="7"/>
       <c r="C38" s="3" t="s">
         <v>95</v>
       </c>
@@ -5433,10 +5442,10 @@
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A39" s="7" t="s">
+      <c r="A39" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="7" t="s">
         <v>96</v>
       </c>
       <c r="C39" t="s">
@@ -5486,8 +5495,8 @@
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A40" s="7"/>
-      <c r="B40" s="5"/>
+      <c r="A40" s="4"/>
+      <c r="B40" s="7"/>
       <c r="C40" t="s">
         <v>98</v>
       </c>
@@ -5535,8 +5544,8 @@
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A41" s="7"/>
-      <c r="B41" s="5"/>
+      <c r="A41" s="4"/>
+      <c r="B41" s="7"/>
       <c r="C41" t="s">
         <v>99</v>
       </c>
@@ -5584,10 +5593,10 @@
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A42" s="7" t="s">
+      <c r="A42" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="7" t="s">
         <v>100</v>
       </c>
       <c r="C42" t="s">
@@ -5637,8 +5646,8 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A43" s="7"/>
-      <c r="B43" s="5"/>
+      <c r="A43" s="4"/>
+      <c r="B43" s="7"/>
       <c r="C43" t="s">
         <v>102</v>
       </c>
@@ -5686,8 +5695,8 @@
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A44" s="7"/>
-      <c r="B44" s="5"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="7"/>
       <c r="C44" t="s">
         <v>103</v>
       </c>
@@ -5736,19 +5745,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="P13:R13"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A18:A20"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="B39:B41"/>
@@ -5759,6 +5755,19 @@
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B30:B32"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="A36:A38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
New asset files and fixes to level unlock and tutorial. New demo release for DevGAMM
</commit_message>
<xml_diff>
--- a/Food Progression.xlsx
+++ b/Food Progression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Nutri Mayhem\NutriCrush-Unity-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE15FB26-A830-4388-8230-F36FDDA13DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A05476-2CE2-473D-9352-44E9549ACBF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{3A71858E-782A-488A-BF56-898FF2A6D53B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="156">
   <si>
     <t>Id</t>
   </si>
@@ -1001,16 +1001,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4015,6 +4015,18 @@
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B3">
@@ -4027,7 +4039,19 @@
         <v>75</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>0.8</v>
+      </c>
+      <c r="G3">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="H3">
+        <v>1.5</v>
+      </c>
+      <c r="I3">
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
@@ -4043,6 +4067,18 @@
       <c r="E4">
         <v>3</v>
       </c>
+      <c r="F4">
+        <v>0.4</v>
+      </c>
+      <c r="G4">
+        <v>9.7000000000000003E-2</v>
+      </c>
+      <c r="H4">
+        <v>0.4</v>
+      </c>
+      <c r="I4">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5">
@@ -4055,7 +4091,19 @@
         <v>25</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>0.3</v>
+      </c>
+      <c r="G5">
+        <v>0.03</v>
+      </c>
+      <c r="H5">
+        <v>1.9</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
@@ -4069,7 +4117,19 @@
         <v>78</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="F6">
+        <v>3.4</v>
+      </c>
+      <c r="G6">
+        <v>6.2E-2</v>
+      </c>
+      <c r="H6">
+        <v>0.6</v>
+      </c>
+      <c r="I6">
+        <v>1.6</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
@@ -4083,7 +4143,19 @@
         <v>34</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>0.4</v>
+      </c>
+      <c r="G7">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="H7">
+        <v>1.7</v>
+      </c>
+      <c r="I7">
+        <v>0.1</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
@@ -4097,16 +4169,19 @@
         <v>18</v>
       </c>
       <c r="E8">
-        <v>3</v>
-      </c>
-      <c r="J8">
-        <v>30</v>
-      </c>
-      <c r="K8" t="s">
-        <v>42</v>
-      </c>
-      <c r="L8">
-        <v>30</v>
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>0.2</v>
+      </c>
+      <c r="G8">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="H8">
+        <v>2.6</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
@@ -4120,7 +4195,19 @@
         <v>17</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>0.2</v>
+      </c>
+      <c r="G9">
+        <v>1E-3</v>
+      </c>
+      <c r="H9">
+        <v>2.5</v>
+      </c>
+      <c r="I9">
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
@@ -4134,7 +4221,19 @@
         <v>45</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10">
+        <v>0.32</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
@@ -4150,6 +4249,18 @@
       <c r="E11">
         <v>3</v>
       </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="H11">
+        <v>5</v>
+      </c>
+      <c r="I11">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12">
@@ -4162,25 +4273,37 @@
         <v>30</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>0.2</v>
+      </c>
+      <c r="G12">
+        <v>0.05</v>
+      </c>
+      <c r="H12">
+        <v>3.4</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5" t="s">
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5" t="s">
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
@@ -4234,10 +4357,10 @@
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C15" t="s">
@@ -4287,8 +4410,8 @@
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A16" s="4"/>
-      <c r="B16" s="7"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="5"/>
       <c r="C16" t="s">
         <v>66</v>
       </c>
@@ -4336,8 +4459,8 @@
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A17" s="4"/>
-      <c r="B17" s="7"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="5"/>
       <c r="C17" t="s">
         <v>67</v>
       </c>
@@ -4385,10 +4508,10 @@
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>68</v>
       </c>
       <c r="C18" t="s">
@@ -4438,8 +4561,8 @@
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A19" s="4"/>
-      <c r="B19" s="7"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="5"/>
       <c r="C19" t="s">
         <v>70</v>
       </c>
@@ -4487,8 +4610,8 @@
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A20" s="4"/>
-      <c r="B20" s="7"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="5"/>
       <c r="C20" t="s">
         <v>71</v>
       </c>
@@ -4536,10 +4659,10 @@
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="5" t="s">
         <v>72</v>
       </c>
       <c r="C21" t="s">
@@ -4589,8 +4712,8 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A22" s="4"/>
-      <c r="B22" s="7"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="5"/>
       <c r="C22" t="s">
         <v>74</v>
       </c>
@@ -4638,8 +4761,8 @@
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A23" s="4"/>
-      <c r="B23" s="7"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="5"/>
       <c r="C23" t="s">
         <v>75</v>
       </c>
@@ -4687,10 +4810,10 @@
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C24" t="s">
@@ -4740,8 +4863,8 @@
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A25" s="4"/>
-      <c r="B25" s="7"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="5"/>
       <c r="C25" t="s">
         <v>78</v>
       </c>
@@ -4789,8 +4912,8 @@
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A26" s="4"/>
-      <c r="B26" s="7"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="5"/>
       <c r="C26" t="s">
         <v>79</v>
       </c>
@@ -4838,10 +4961,10 @@
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C27" t="s">
@@ -4891,8 +5014,8 @@
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A28" s="4"/>
-      <c r="B28" s="7"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="5"/>
       <c r="C28" t="s">
         <v>82</v>
       </c>
@@ -4940,8 +5063,8 @@
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A29" s="4"/>
-      <c r="B29" s="7"/>
+      <c r="A29" s="7"/>
+      <c r="B29" s="5"/>
       <c r="C29" t="s">
         <v>83</v>
       </c>
@@ -4989,10 +5112,10 @@
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="5" t="s">
         <v>84</v>
       </c>
       <c r="C30" t="s">
@@ -5042,8 +5165,8 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A31" s="4"/>
-      <c r="B31" s="7"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="5"/>
       <c r="C31" t="s">
         <v>86</v>
       </c>
@@ -5091,8 +5214,8 @@
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A32" s="4"/>
-      <c r="B32" s="7"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="5"/>
       <c r="C32" t="s">
         <v>87</v>
       </c>
@@ -5140,10 +5263,10 @@
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C33" t="s">
@@ -5193,8 +5316,8 @@
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A34" s="4"/>
-      <c r="B34" s="6"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="4"/>
       <c r="C34" t="s">
         <v>90</v>
       </c>
@@ -5242,8 +5365,8 @@
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A35" s="4"/>
-      <c r="B35" s="6"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="4"/>
       <c r="C35" t="s">
         <v>91</v>
       </c>
@@ -5291,10 +5414,10 @@
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="5" t="s">
         <v>92</v>
       </c>
       <c r="C36" t="s">
@@ -5344,8 +5467,8 @@
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A37" s="4"/>
-      <c r="B37" s="7"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="5"/>
       <c r="C37" t="s">
         <v>94</v>
       </c>
@@ -5393,8 +5516,8 @@
       </c>
     </row>
     <row r="38" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="4"/>
-      <c r="B38" s="7"/>
+      <c r="A38" s="7"/>
+      <c r="B38" s="5"/>
       <c r="C38" s="3" t="s">
         <v>95</v>
       </c>
@@ -5442,10 +5565,10 @@
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="5" t="s">
         <v>96</v>
       </c>
       <c r="C39" t="s">
@@ -5495,8 +5618,8 @@
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A40" s="4"/>
-      <c r="B40" s="7"/>
+      <c r="A40" s="7"/>
+      <c r="B40" s="5"/>
       <c r="C40" t="s">
         <v>98</v>
       </c>
@@ -5544,8 +5667,8 @@
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A41" s="4"/>
-      <c r="B41" s="7"/>
+      <c r="A41" s="7"/>
+      <c r="B41" s="5"/>
       <c r="C41" t="s">
         <v>99</v>
       </c>
@@ -5593,10 +5716,10 @@
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="5" t="s">
         <v>100</v>
       </c>
       <c r="C42" t="s">
@@ -5646,8 +5769,8 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A43" s="4"/>
-      <c r="B43" s="7"/>
+      <c r="A43" s="7"/>
+      <c r="B43" s="5"/>
       <c r="C43" t="s">
         <v>102</v>
       </c>
@@ -5695,8 +5818,8 @@
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A44" s="4"/>
-      <c r="B44" s="7"/>
+      <c r="A44" s="7"/>
+      <c r="B44" s="5"/>
       <c r="C44" t="s">
         <v>103</v>
       </c>
@@ -5745,6 +5868,19 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="P13:R13"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A20"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="B39:B41"/>
@@ -5755,19 +5891,6 @@
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B30:B32"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="P13:R13"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A36:A38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>